<commit_message>
OC2 object detector half-ly done
</commit_message>
<xml_diff>
--- a/huskylens.xlsx
+++ b/huskylens.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/likayauelwin/Documents/GitHub/2025-WRO-Future-Engineer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D5DB6C15-3718-054D-BB30-B58D66AFCA7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12DD63F9-A1FB-7442-8802-917837B83FC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="760" windowWidth="28040" windowHeight="17240" xr2:uid="{50C2FC8F-A61D-EA40-BD48-FD46821D1210}"/>
   </bookViews>
@@ -16,8 +16,10 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlchart.v2.0" hidden="1">Sheet1!$D$18:$D$23</definedName>
-    <definedName name="_xlchart.v2.1" hidden="1">Sheet1!$E$18:$E$23</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">Sheet1!$E$35:$E$41</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$F$35:$F$41</definedName>
+    <definedName name="_xlchart.v2.2" hidden="1">Sheet1!$E$35:$E$41</definedName>
+    <definedName name="_xlchart.v2.3" hidden="1">Sheet1!$F$35:$F$41</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
   <si>
     <t>Area</t>
   </si>
@@ -59,15 +61,31 @@
   <si>
     <t>Block at right case:</t>
   </si>
+  <si>
+    <t>y-pos</t>
+  </si>
+  <si>
+    <t>danger</t>
+  </si>
+  <si>
+    <t>real dist (cm)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -93,8 +111,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -249,22 +268,22 @@
                   <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>14</c:v>
+                  <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>22</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>27</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>61</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -276,25 +295,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>125</c:v>
+                  <c:v>107</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>119</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>110</c:v>
+                  <c:v>87</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>101</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>91</c:v>
+                  <c:v>43</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>84</c:v>
+                  <c:v>39</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>58</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -620,22 +639,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>4</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>9</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>13</c:v>
+                  <c:v>23</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>18</c:v>
+                  <c:v>40</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -647,22 +666,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>193</c:v>
+                  <c:v>215</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>198</c:v>
+                  <c:v>224</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>208</c:v>
+                  <c:v>233</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>213</c:v>
+                  <c:v>245</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>221</c:v>
+                  <c:v>265</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>229</c:v>
+                  <c:v>284</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -854,6 +873,330 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$E$35:$E$41</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>25</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$F$35:$F$41</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>160</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>140</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>130</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>110</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>100</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-80E7-A545-80F4-0CCCAFB8BBFB}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="983326944"/>
+        <c:axId val="667356400"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="983326944"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="667356400"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="667356400"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="983326944"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -934,6 +1277,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -1451,6 +1834,522 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2007,15 +2906,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>675555</xdr:colOff>
+      <xdr:colOff>523155</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>154534</xdr:rowOff>
+      <xdr:rowOff>144374</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>316967</xdr:colOff>
+      <xdr:colOff>164567</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>58911</xdr:rowOff>
+      <xdr:rowOff>48751</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2042,16 +2941,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>101600</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>135467</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>160867</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>694266</xdr:colOff>
-      <xdr:row>53</xdr:row>
-      <xdr:rowOff>110170</xdr:rowOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>287866</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>135570</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2074,14 +2973,50 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="931333" y="5825067"/>
-          <a:ext cx="7772400" cy="5054703"/>
+          <a:off x="13106400" y="973667"/>
+          <a:ext cx="7831666" cy="5054703"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>538480</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>172720</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>193040</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9FC1428A-713B-4C2E-F76D-E5C327D046E8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -2404,10 +3339,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4ABAF86-B548-3B4C-9384-3449F00EA32C}">
-  <dimension ref="C1:E25"/>
+  <dimension ref="C1:G41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="28.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:5" x14ac:dyDescent="0.2">
@@ -2429,15 +3365,15 @@
         <v>4</v>
       </c>
       <c r="E2">
-        <v>125</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D3">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E3">
-        <v>119</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="3:5" x14ac:dyDescent="0.2">
@@ -2445,39 +3381,39 @@
         <v>9</v>
       </c>
       <c r="E4">
-        <v>110</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D5">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E5">
-        <v>101</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D6">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E6">
-        <v>91</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D7">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E7">
-        <v>84</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D8">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="E8">
-        <v>58</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="3:5" x14ac:dyDescent="0.2">
@@ -2496,66 +3432,123 @@
         <v>3</v>
       </c>
       <c r="D18">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E18">
-        <v>193</v>
+        <v>215</v>
       </c>
     </row>
     <row r="19" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D19">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E19">
-        <v>198</v>
+        <v>224</v>
       </c>
     </row>
     <row r="20" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D20">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E20">
-        <v>208</v>
+        <v>233</v>
       </c>
     </row>
     <row r="21" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D21">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E21">
-        <v>213</v>
+        <v>245</v>
       </c>
     </row>
     <row r="22" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D22">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="E22">
-        <v>221</v>
+        <v>265</v>
       </c>
     </row>
     <row r="23" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D23">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="E23">
-        <v>229</v>
+        <v>284</v>
       </c>
     </row>
-    <row r="24" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="D24">
-        <v>29</v>
-      </c>
-      <c r="E24">
-        <v>246</v>
+    <row r="34" spans="4:7" x14ac:dyDescent="0.2">
+      <c r="E34" t="s">
+        <v>8</v>
+      </c>
+      <c r="F34" t="s">
+        <v>6</v>
+      </c>
+      <c r="G34" t="s">
+        <v>0</v>
       </c>
     </row>
-    <row r="25" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="D25">
-        <v>53</v>
-      </c>
-      <c r="E25">
-        <v>276</v>
+    <row r="35" spans="4:7" x14ac:dyDescent="0.2">
+      <c r="D35" t="s">
+        <v>7</v>
+      </c>
+      <c r="E35" s="1">
+        <v>70</v>
+      </c>
+      <c r="F35" s="1">
+        <v>160</v>
+      </c>
+      <c r="G35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="4:7" x14ac:dyDescent="0.2">
+      <c r="E36">
+        <v>60</v>
+      </c>
+      <c r="F36">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="37" spans="4:7" x14ac:dyDescent="0.2">
+      <c r="E37">
+        <v>50</v>
+      </c>
+      <c r="F37">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="38" spans="4:7" x14ac:dyDescent="0.2">
+      <c r="E38">
+        <v>45</v>
+      </c>
+      <c r="F38">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="39" spans="4:7" x14ac:dyDescent="0.2">
+      <c r="E39">
+        <v>40</v>
+      </c>
+      <c r="F39">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="40" spans="4:7" x14ac:dyDescent="0.2">
+      <c r="E40">
+        <v>35</v>
+      </c>
+      <c r="F40">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="41" spans="4:7" x14ac:dyDescent="0.2">
+      <c r="E41">
+        <v>25</v>
+      </c>
+      <c r="F41">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Forgot to push this
</commit_message>
<xml_diff>
--- a/huskylens.xlsx
+++ b/huskylens.xlsx
@@ -8,19 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/likayauelwin/Documents/GitHub/2025-WRO-Future-Engineer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12DD63F9-A1FB-7442-8802-917837B83FC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{363A264B-24E4-354F-A7E3-E95A33127133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="760" windowWidth="28040" windowHeight="17240" xr2:uid="{50C2FC8F-A61D-EA40-BD48-FD46821D1210}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Sheet1!$E$35:$E$41</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$F$35:$F$41</definedName>
-    <definedName name="_xlchart.v2.2" hidden="1">Sheet1!$E$35:$E$41</definedName>
-    <definedName name="_xlchart.v2.3" hidden="1">Sheet1!$F$35:$F$41</definedName>
-  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">

</xml_diff>

<commit_message>
Not yet finished refractoring
</commit_message>
<xml_diff>
--- a/huskylens.xlsx
+++ b/huskylens.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/likayauelwin/Documents/GitHub/2025-WRO-Future-Engineer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF3E6AA5-3252-8949-A7D6-6FAE066CDFE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{479A67CD-FA4F-0C42-9C7F-95D7C2EA5D25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="760" windowWidth="28040" windowHeight="17240" xr2:uid="{50C2FC8F-A61D-EA40-BD48-FD46821D1210}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>